<commit_message>
[Added] Completed login module test cases
</commit_message>
<xml_diff>
--- a/data/Customer-Panel.xlsx
+++ b/data/Customer-Panel.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>email</t>
   </si>
@@ -23,6 +23,12 @@
   </si>
   <si>
     <t>Relinns@321</t>
+  </si>
+  <si>
+    <t>gaurangi</t>
+  </si>
+  <si>
+    <t>Relinns@123</t>
   </si>
 </sst>
 </file>
@@ -299,6 +305,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>